<commit_message>
Regenerate Section 32 report after independent audit
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/GPT-5-6-SOL/Section_32-11N-25W_Beckham_Co_Diversified_Cursory_Report_GPT-5-6-SOL_TOURNAMENT_20260806_CONFLICT_ASSUMPTION_REGISTER.xlsx
+++ b/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/GPT-5-6-SOL/Section_32-11N-25W_Beckham_Co_Diversified_Cursory_Report_GPT-5-6-SOL_TOURNAMENT_20260806_CONFLICT_ASSUMPTION_REGISTER.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -607,7 +607,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Diversified Production LLC is the latest supported named claimant, not a proven 640-acre/100% owner.</t>
+          <t>Diversified is the last claimant supported by the reviewed 2400 schedule, not a confirmed current or 640-acre/100% owner.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -802,6 +802,60 @@
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Map each operative modern schedule lease-by-lease.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>C-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Bk 2434/751 may convey Diversified/DP Legacy Central interests to Teocalli after the reviewed-title cutoff.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>V10 county-index lead; recorded face and schedule unavailable</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Diversified is described only as the last claimant supported by the reviewed 2400 schedule. Current claimant status is expressly unconfirmed.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>CRITICAL — read 2434/751 first and determine whether Section 32/OK48147.001.1 is included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>C-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Viersen OGL 332/74-75 has no lessor-mineral vesting crosswalk to the estimated NE/4 owners.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>V10 lease-to-owner coverage audit; OGL face reviewed</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Coverage gap is visible on OGL and Tract 1; no current leasehold conclusion is drawn.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Establish Viersen lessor vesting and reconcile it to the NE/4 title schedule.</t>
         </is>
       </c>
     </row>

</xml_diff>